<commit_message>
sync: 2026-04-14 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dra-vanessa-soares/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dra-vanessa-soares/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -114,7 +114,13 @@
     <t>[HARMONIZAÇÃO MASCULINA] [SYRA] [WHATSAPP]</t>
   </si>
   <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
     <t>11/11/2025</t>
+  </si>
+  <si>
+    <t>✅ Ativa</t>
   </si>
   <si>
     <t>ID do Adset</t>
@@ -176,7 +182,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +204,11 @@
         <fgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -211,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -222,6 +233,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,8 +834,8 @@
       <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>17</v>
+      <c r="C6" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>18</v>
@@ -832,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G6" s="6">
         <v>0</v>
@@ -859,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -888,13 +900,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -903,7 +915,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -918,30 +930,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
-        <v>39</v>
-      </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -959,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -986,19 +998,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -1016,24 +1028,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1048,10 +1060,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>